<commit_message>
Benennung der Assets an prod  System angepasst. Benennung und Beschreibung der Aktivittäten
</commit_message>
<xml_diff>
--- a/performer/Data/Config.xlsx
+++ b/performer/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KM\KM6\KM61_neu\15_RPA\02_Beurteilungsdaten_übertragen\rpa005_TBÜ_Performer_V2\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KM\KM6\KM61_neu\15_RPA\02_Beurteilungsdaten_übertragen\repo\performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FD1B54C-2876-406C-9C4E-A0FFD4208ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9E477A-2B1D-4491-ABEA-1D71D56E5AD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29355" yWindow="-3720" windowWidth="29100" windowHeight="15765" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-51600" yWindow="4590" windowWidth="22065" windowHeight="20745" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="64">
   <si>
     <t>Name</t>
   </si>
@@ -189,9 +189,6 @@
     <t>rpa005_SAP_Client</t>
   </si>
   <si>
-    <t>Test/POR/rpa005_TBÜ</t>
-  </si>
-  <si>
     <t>rpa005_JsonNewFolderPath</t>
   </si>
   <si>
@@ -210,13 +207,16 @@
     <t>rpa005_SAP-Account_K31</t>
   </si>
   <si>
-    <t>rpa005_TestGroup_Mailbox</t>
-  </si>
-  <si>
-    <t>rpa005_Test_VersandMail</t>
-  </si>
-  <si>
     <t>rpa005_LogFileFolderPath</t>
+  </si>
+  <si>
+    <t>rpa005_Bot_Email_Address</t>
+  </si>
+  <si>
+    <t>rpa005_Email_Group_Mailbox</t>
+  </si>
+  <si>
+    <t>rpa005_Email_Exception_Mailbox</t>
   </si>
 </sst>
 </file>
@@ -649,10 +649,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>59</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>2</v>
@@ -696,9 +696,6 @@
       <c r="A3" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="D3" s="6" t="s">
         <v>31</v>
       </c>
@@ -720,7 +717,7 @@
         <v>44</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" s="3"/>
     </row>
@@ -1747,10 +1744,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -2930,7 +2927,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z999"/>
+  <dimension ref="A1:Z998"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="5" customWidth="1"/>
@@ -3042,26 +3039,26 @@
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -3089,22 +3086,29 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A16" s="10" t="s">
-        <v>62</v>
+      <c r="A16" s="5" t="s">
+        <v>60</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A18" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B18" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
@@ -4085,7 +4089,6 @@
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add new cleaned current state
</commit_message>
<xml_diff>
--- a/performer/Data/Config.xlsx
+++ b/performer/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KM\KM6\KM61_neu\15_RPA\02_Beurteilungsdaten_übertragen\rpa005_TBÜ_Performer_V2\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KM\KM6\KM61_neu\15_RPA\02_Beurteilungsdaten_übertragen\repo\performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FD1B54C-2876-406C-9C4E-A0FFD4208ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553EAC79-474E-4A6E-8DE0-7D2DC0B41B4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29355" yWindow="-3720" windowWidth="29100" windowHeight="15765" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="60">
   <si>
     <t>Name</t>
   </si>
@@ -156,74 +156,62 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
+    <t>rpa005_EmailSmtpPort</t>
+  </si>
+  <si>
+    <t>rpa005_EmailSmtpServer</t>
+  </si>
+  <si>
+    <t>rpa005_SAP_ConnectionName</t>
+  </si>
+  <si>
+    <t>rpa005_SAP_FirstTransaction</t>
+  </si>
+  <si>
+    <t>rpa005_FTP_Client_Url</t>
+  </si>
+  <si>
+    <t>rpa005_SAP_Language</t>
+  </si>
+  <si>
+    <t>rpa005_SAP_Client</t>
+  </si>
+  <si>
+    <t>rpa005_JsonNewFolderPath</t>
+  </si>
+  <si>
+    <t>rpa005_JsonProcessedFolderPath</t>
+  </si>
+  <si>
+    <t>rpa005_JsonErrorFolderPath</t>
+  </si>
+  <si>
+    <t>Test Value</t>
+  </si>
+  <si>
+    <t>Prod Value</t>
+  </si>
+  <si>
+    <t>rpa005_LogFileFolderPath</t>
+  </si>
+  <si>
+    <t>rpa005_Bot_Email_Address</t>
+  </si>
+  <si>
+    <t>rpa005_Email_Group_Mailbox</t>
+  </si>
+  <si>
+    <t>rpa005_Email_Exception_Mailbox</t>
+  </si>
+  <si>
     <t>rpa005_Beurteilungsdaten_übertragen</t>
-  </si>
-  <si>
-    <t>SAP_CredentialAssetName</t>
-  </si>
-  <si>
-    <t>TMS_FTP_CredentialAssetName</t>
-  </si>
-  <si>
-    <t>rpa005_TMS_FTP_Account</t>
-  </si>
-  <si>
-    <t>rpa005_EmailSmtpPort</t>
-  </si>
-  <si>
-    <t>rpa005_EmailSmtpServer</t>
-  </si>
-  <si>
-    <t>rpa005_SAP_ConnectionName</t>
-  </si>
-  <si>
-    <t>rpa005_SAP_FirstTransaction</t>
-  </si>
-  <si>
-    <t>rpa005_FTP_Client_Url</t>
-  </si>
-  <si>
-    <t>rpa005_SAP_Language</t>
-  </si>
-  <si>
-    <t>rpa005_SAP_Client</t>
-  </si>
-  <si>
-    <t>Test/POR/rpa005_TBÜ</t>
-  </si>
-  <si>
-    <t>rpa005_JsonNewFolderPath</t>
-  </si>
-  <si>
-    <t>rpa005_JsonProcessedFolderPath</t>
-  </si>
-  <si>
-    <t>rpa005_JsonErrorFolderPath</t>
-  </si>
-  <si>
-    <t>Test Value</t>
-  </si>
-  <si>
-    <t>Prod Value</t>
-  </si>
-  <si>
-    <t>rpa005_SAP-Account_K31</t>
-  </si>
-  <si>
-    <t>rpa005_TestGroup_Mailbox</t>
-  </si>
-  <si>
-    <t>rpa005_Test_VersandMail</t>
-  </si>
-  <si>
-    <t>rpa005_LogFileFolderPath</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -281,6 +269,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -302,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -320,6 +314,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -649,10 +644,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>2</v>
@@ -685,8 +680,11 @@
       <c r="A2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>43</v>
+      <c r="B2" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>59</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>21</v>
@@ -695,9 +693,6 @@
     <row r="3" spans="1:27" ht="45">
       <c r="A3" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>54</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>31</v>
@@ -716,21 +711,11 @@
       </c>
     </row>
     <row r="6" spans="1:27" ht="14.25" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:27" ht="14.25" customHeight="1">
-      <c r="A7" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>46</v>
-      </c>
+      <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:27" ht="14.25" customHeight="1"/>
@@ -1747,10 +1732,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -2930,7 +2915,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z999"/>
+  <dimension ref="A1:Z998"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="5" customWidth="1"/>
@@ -2978,133 +2963,140 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" s="8" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" s="9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" s="9" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A16" s="10" t="s">
-        <v>62</v>
+      <c r="A16" s="5" t="s">
+        <v>55</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="18" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A18" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
@@ -4085,7 +4077,6 @@
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>